<commit_message>
Cleaned up for first commit on branch
</commit_message>
<xml_diff>
--- a/Timesheet Template/Excel Test File.xlsx
+++ b/Timesheet Template/Excel Test File.xlsx
@@ -825,7 +825,7 @@
       <c r="F16" s="1" t="n"/>
       <c r="G16" s="32" t="inlineStr">
         <is>
-          <t>5/15/2025</t>
+          <t>1/6/2025</t>
         </is>
       </c>
       <c r="H16" s="31" t="n"/>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>01/09/2025</t>
+          <t>01/10/2025</t>
         </is>
       </c>
       <c r="F41" s="31" t="n"/>
@@ -1576,7 +1576,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>C:/Users/SharikMahmood/OneDrive - Creative Electron Inc/Desktop/New folder</t>
+          <t>C:\Users\SharikMahmood\Documents</t>
         </is>
       </c>
     </row>

</xml_diff>